<commit_message>
Matrices en excel cada instancia
</commit_message>
<xml_diff>
--- a/output/resultado_resumen_final.xlsx
+++ b/output/resultado_resumen_final.xlsx
@@ -427,7 +427,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -439,13 +439,13 @@
         <v>2</v>
       </c>
       <c r="G2">
-        <v>0.08699999999999999</v>
+        <v>0.049</v>
       </c>
       <c r="H2">
-        <v>3.802</v>
+        <v>2.689</v>
       </c>
       <c r="I2">
-        <v>2.572</v>
+        <v>3.318</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -453,7 +453,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -465,13 +465,13 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <v>0.081</v>
+        <v>0.043</v>
       </c>
       <c r="H3">
-        <v>3.571</v>
+        <v>2.52</v>
       </c>
       <c r="I3">
-        <v>2.688</v>
+        <v>3.389</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -479,7 +479,7 @@
         <v>1</v>
       </c>
       <c r="B4">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -488,19 +488,19 @@
         <v>14</v>
       </c>
       <c r="E4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4">
-        <v>1.1693</v>
+        <v>1.2573</v>
       </c>
       <c r="G4">
-        <v>0.185</v>
+        <v>0.066</v>
       </c>
       <c r="H4">
-        <v>2.589</v>
+        <v>1.89</v>
       </c>
       <c r="I4">
-        <v>1.236</v>
+        <v>2.122</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -508,7 +508,7 @@
         <v>1</v>
       </c>
       <c r="B5">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
@@ -520,13 +520,13 @@
         <v>2</v>
       </c>
       <c r="G5">
-        <v>0.079</v>
+        <v>0.045</v>
       </c>
       <c r="H5">
-        <v>3.509</v>
+        <v>2.576</v>
       </c>
       <c r="I5">
-        <v>2.707</v>
+        <v>3.392</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -534,7 +534,7 @@
         <v>1</v>
       </c>
       <c r="B6">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
         <v>10</v>
@@ -546,13 +546,13 @@
         <v>2</v>
       </c>
       <c r="G6">
-        <v>0.082</v>
+        <v>0.053</v>
       </c>
       <c r="H6">
-        <v>3.601</v>
+        <v>2.545</v>
       </c>
       <c r="I6">
-        <v>2.604</v>
+        <v>3.157</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -560,7 +560,7 @@
         <v>1</v>
       </c>
       <c r="B7">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
@@ -569,19 +569,19 @@
         <v>14</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>1.2071</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>0.094</v>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>2.219</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>1.839</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -589,7 +589,7 @@
         <v>1</v>
       </c>
       <c r="B8">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C8" t="s">
         <v>11</v>
@@ -601,13 +601,13 @@
         <v>2</v>
       </c>
       <c r="G8">
-        <v>0.077</v>
+        <v>0.06</v>
       </c>
       <c r="H8">
-        <v>3.464</v>
+        <v>2.907</v>
       </c>
       <c r="I8">
-        <v>2.733</v>
+        <v>2.942</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -615,7 +615,7 @@
         <v>1</v>
       </c>
       <c r="B9">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
@@ -627,13 +627,13 @@
         <v>2</v>
       </c>
       <c r="G9">
-        <v>0.082</v>
+        <v>0.058</v>
       </c>
       <c r="H9">
-        <v>3.63</v>
+        <v>2.838</v>
       </c>
       <c r="I9">
-        <v>2.594</v>
+        <v>2.865</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -641,7 +641,7 @@
         <v>1</v>
       </c>
       <c r="B10">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
         <v>11</v>
@@ -653,16 +653,16 @@
         <v>2</v>
       </c>
       <c r="F10">
-        <v>1.1362</v>
+        <v>1.2223</v>
       </c>
       <c r="G10">
-        <v>0.118</v>
+        <v>0.111</v>
       </c>
       <c r="H10">
-        <v>1.84</v>
+        <v>2.344</v>
       </c>
       <c r="I10">
-        <v>1.468</v>
+        <v>1.681</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -670,7 +670,7 @@
         <v>2</v>
       </c>
       <c r="B11">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
@@ -682,13 +682,13 @@
         <v>2</v>
       </c>
       <c r="G11">
-        <v>0.081</v>
+        <v>0.04</v>
       </c>
       <c r="H11">
-        <v>3.69</v>
+        <v>2.834</v>
       </c>
       <c r="I11">
-        <v>2.635</v>
+        <v>3.737</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -696,7 +696,7 @@
         <v>2</v>
       </c>
       <c r="B12">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
         <v>9</v>
@@ -705,16 +705,16 @@
         <v>13</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G12">
-        <v>0.077</v>
+        <v>0.045</v>
       </c>
       <c r="H12">
-        <v>3.3</v>
+        <v>2.686</v>
       </c>
       <c r="I12">
-        <v>2.312</v>
+        <v>3.752</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -722,7 +722,7 @@
         <v>2</v>
       </c>
       <c r="B13">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
         <v>9</v>
@@ -731,19 +731,19 @@
         <v>14</v>
       </c>
       <c r="E13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F13">
-        <v>1.1878</v>
+        <v>1.3778</v>
       </c>
       <c r="G13">
-        <v>0.142</v>
+        <v>0.039</v>
       </c>
       <c r="H13">
-        <v>3.458</v>
+        <v>1.782</v>
       </c>
       <c r="I13">
-        <v>1.782</v>
+        <v>2.426</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -751,7 +751,7 @@
         <v>2</v>
       </c>
       <c r="B14">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C14" t="s">
         <v>10</v>
@@ -763,13 +763,13 @@
         <v>2</v>
       </c>
       <c r="G14">
-        <v>0.056</v>
+        <v>0.043</v>
       </c>
       <c r="H14">
-        <v>2.815</v>
+        <v>2.937</v>
       </c>
       <c r="I14">
-        <v>3.049</v>
+        <v>3.676</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -777,7 +777,7 @@
         <v>2</v>
       </c>
       <c r="B15">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C15" t="s">
         <v>10</v>
@@ -789,13 +789,13 @@
         <v>2</v>
       </c>
       <c r="G15">
-        <v>0.065</v>
+        <v>0.041</v>
       </c>
       <c r="H15">
-        <v>3.062</v>
+        <v>2.618</v>
       </c>
       <c r="I15">
-        <v>2.958</v>
+        <v>3.787</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -803,7 +803,7 @@
         <v>2</v>
       </c>
       <c r="B16">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
         <v>10</v>
@@ -812,19 +812,19 @@
         <v>14</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F16">
-        <v>1.1239</v>
+        <v>1.2927</v>
       </c>
       <c r="G16">
-        <v>0.136</v>
+        <v>0.046</v>
       </c>
       <c r="H16">
-        <v>2.813</v>
+        <v>1.69</v>
       </c>
       <c r="I16">
-        <v>1.767</v>
+        <v>2.097</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -832,7 +832,7 @@
         <v>2</v>
       </c>
       <c r="B17">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C17" t="s">
         <v>11</v>
@@ -844,13 +844,13 @@
         <v>2</v>
       </c>
       <c r="G17">
-        <v>0.07099999999999999</v>
+        <v>0.044</v>
       </c>
       <c r="H17">
-        <v>3.141</v>
+        <v>2.899</v>
       </c>
       <c r="I17">
-        <v>2.547</v>
+        <v>3.694</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -858,7 +858,7 @@
         <v>2</v>
       </c>
       <c r="B18">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C18" t="s">
         <v>11</v>
@@ -870,13 +870,13 @@
         <v>2</v>
       </c>
       <c r="G18">
-        <v>0.08400000000000001</v>
+        <v>0.05</v>
       </c>
       <c r="H18">
-        <v>3.177</v>
+        <v>3.087</v>
       </c>
       <c r="I18">
-        <v>2.584</v>
+        <v>3.485</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -884,7 +884,7 @@
         <v>2</v>
       </c>
       <c r="B19">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C19" t="s">
         <v>11</v>
@@ -893,19 +893,19 @@
         <v>14</v>
       </c>
       <c r="E19">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F19">
-        <v>1.1227</v>
+        <v>1.2873</v>
       </c>
       <c r="G19">
-        <v>0.212</v>
+        <v>0.056</v>
       </c>
       <c r="H19">
-        <v>3.4</v>
+        <v>2.151</v>
       </c>
       <c r="I19">
-        <v>1.263</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -913,7 +913,7 @@
         <v>3</v>
       </c>
       <c r="B20">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="C20" t="s">
         <v>9</v>
@@ -925,13 +925,13 @@
         <v>2</v>
       </c>
       <c r="G20">
-        <v>0.032</v>
+        <v>0.058</v>
       </c>
       <c r="H20">
-        <v>3.786</v>
+        <v>3.043</v>
       </c>
       <c r="I20">
-        <v>4.383</v>
+        <v>3.076</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -939,7 +939,7 @@
         <v>3</v>
       </c>
       <c r="B21">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="C21" t="s">
         <v>9</v>
@@ -948,16 +948,16 @@
         <v>13</v>
       </c>
       <c r="E21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G21">
-        <v>0.036</v>
+        <v>0.049</v>
       </c>
       <c r="H21">
-        <v>3.568</v>
+        <v>2.661</v>
       </c>
       <c r="I21">
-        <v>4.534</v>
+        <v>2.743</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -965,7 +965,7 @@
         <v>3</v>
       </c>
       <c r="B22">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="C22" t="s">
         <v>9</v>
@@ -974,19 +974,19 @@
         <v>14</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>1.2398</v>
       </c>
       <c r="G22">
-        <v>0</v>
+        <v>0.126</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>2.397</v>
       </c>
       <c r="I22">
-        <v>0</v>
+        <v>1.682</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -994,7 +994,7 @@
         <v>3</v>
       </c>
       <c r="B23">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="C23" t="s">
         <v>10</v>
@@ -1006,13 +1006,13 @@
         <v>2</v>
       </c>
       <c r="G23">
-        <v>0.03</v>
+        <v>0.074</v>
       </c>
       <c r="H23">
-        <v>3.562</v>
+        <v>3.248</v>
       </c>
       <c r="I23">
-        <v>4.188</v>
+        <v>2.859</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1020,7 +1020,7 @@
         <v>3</v>
       </c>
       <c r="B24">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="C24" t="s">
         <v>10</v>
@@ -1032,13 +1032,13 @@
         <v>2</v>
       </c>
       <c r="G24">
-        <v>0.018</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H24">
-        <v>2.76</v>
+        <v>2.71</v>
       </c>
       <c r="I24">
-        <v>3.882</v>
+        <v>2.681</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1046,7 +1046,7 @@
         <v>3</v>
       </c>
       <c r="B25">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="C25" t="s">
         <v>10</v>
@@ -1055,19 +1055,19 @@
         <v>14</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F25">
-        <v>0</v>
+        <v>1.1394</v>
       </c>
       <c r="G25">
-        <v>0</v>
+        <v>0.073</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>2.087</v>
       </c>
       <c r="I25">
-        <v>0</v>
+        <v>1.863</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1075,7 +1075,7 @@
         <v>3</v>
       </c>
       <c r="B26">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="C26" t="s">
         <v>11</v>
@@ -1087,13 +1087,13 @@
         <v>2</v>
       </c>
       <c r="G26">
-        <v>0.027</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H26">
-        <v>3.342</v>
+        <v>3.157</v>
       </c>
       <c r="I26">
-        <v>4.508</v>
+        <v>2.999</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1101,7 +1101,7 @@
         <v>3</v>
       </c>
       <c r="B27">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="C27" t="s">
         <v>11</v>
@@ -1113,13 +1113,13 @@
         <v>2</v>
       </c>
       <c r="G27">
-        <v>0.024</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="H27">
-        <v>3.222</v>
+        <v>2.963</v>
       </c>
       <c r="I27">
-        <v>4.276</v>
+        <v>2.816</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1127,7 +1127,7 @@
         <v>3</v>
       </c>
       <c r="B28">
-        <v>76</v>
+        <v>31</v>
       </c>
       <c r="C28" t="s">
         <v>11</v>
@@ -1136,19 +1136,19 @@
         <v>14</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>1.152</v>
       </c>
       <c r="G28">
-        <v>0</v>
+        <v>0.118</v>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>2.576</v>
       </c>
       <c r="I28">
-        <v>0</v>
+        <v>1.621</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1156,7 +1156,7 @@
         <v>4</v>
       </c>
       <c r="B29">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C29" t="s">
         <v>9</v>
@@ -1165,16 +1165,16 @@
         <v>12</v>
       </c>
       <c r="E29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G29">
-        <v>0.1</v>
+        <v>0.08</v>
       </c>
       <c r="H29">
-        <v>2.887</v>
+        <v>3.196</v>
       </c>
       <c r="I29">
-        <v>1.967</v>
+        <v>2.607</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1182,7 +1182,7 @@
         <v>4</v>
       </c>
       <c r="B30">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C30" t="s">
         <v>9</v>
@@ -1191,16 +1191,16 @@
         <v>13</v>
       </c>
       <c r="E30">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G30">
-        <v>0.08500000000000001</v>
+        <v>0.096</v>
       </c>
       <c r="H30">
-        <v>2.678</v>
+        <v>3.297</v>
       </c>
       <c r="I30">
-        <v>2.477</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1208,7 +1208,7 @@
         <v>4</v>
       </c>
       <c r="B31">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C31" t="s">
         <v>9</v>
@@ -1220,16 +1220,16 @@
         <v>2</v>
       </c>
       <c r="F31">
-        <v>1.049</v>
+        <v>1.0813</v>
       </c>
       <c r="G31">
-        <v>0.179</v>
+        <v>0.172</v>
       </c>
       <c r="H31">
-        <v>2.85</v>
+        <v>2.519</v>
       </c>
       <c r="I31">
-        <v>1.363</v>
+        <v>1.358</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -1237,7 +1237,7 @@
         <v>4</v>
       </c>
       <c r="B32">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C32" t="s">
         <v>10</v>
@@ -1249,13 +1249,13 @@
         <v>2</v>
       </c>
       <c r="G32">
-        <v>0.101</v>
+        <v>0.082</v>
       </c>
       <c r="H32">
-        <v>3.213</v>
+        <v>3.162</v>
       </c>
       <c r="I32">
-        <v>2.29</v>
+        <v>2.581</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -1263,7 +1263,7 @@
         <v>4</v>
       </c>
       <c r="B33">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C33" t="s">
         <v>10</v>
@@ -1272,16 +1272,16 @@
         <v>13</v>
       </c>
       <c r="E33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G33">
-        <v>0.099</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="H33">
-        <v>2.893</v>
+        <v>3.04</v>
       </c>
       <c r="I33">
-        <v>1.914</v>
+        <v>2.739</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -1289,7 +1289,7 @@
         <v>4</v>
       </c>
       <c r="B34">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C34" t="s">
         <v>10</v>
@@ -1298,19 +1298,19 @@
         <v>14</v>
       </c>
       <c r="E34">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F34">
-        <v>0</v>
+        <v>1.0453</v>
       </c>
       <c r="G34">
-        <v>0</v>
+        <v>0.237</v>
       </c>
       <c r="H34">
-        <v>0</v>
+        <v>3.21</v>
       </c>
       <c r="I34">
-        <v>0</v>
+        <v>1.112</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -1318,7 +1318,7 @@
         <v>4</v>
       </c>
       <c r="B35">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C35" t="s">
         <v>11</v>
@@ -1330,13 +1330,13 @@
         <v>2</v>
       </c>
       <c r="G35">
-        <v>0.08400000000000001</v>
+        <v>0.064</v>
       </c>
       <c r="H35">
-        <v>2.815</v>
+        <v>2.742</v>
       </c>
       <c r="I35">
-        <v>2.41</v>
+        <v>2.887</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -1344,7 +1344,7 @@
         <v>4</v>
       </c>
       <c r="B36">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C36" t="s">
         <v>11</v>
@@ -1353,16 +1353,16 @@
         <v>13</v>
       </c>
       <c r="E36">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G36">
-        <v>0.093</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="H36">
-        <v>2.753</v>
+        <v>2.63</v>
       </c>
       <c r="I36">
-        <v>2.034</v>
+        <v>2.002</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -1370,7 +1370,7 @@
         <v>4</v>
       </c>
       <c r="B37">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C37" t="s">
         <v>11</v>
@@ -1379,19 +1379,19 @@
         <v>14</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F37">
-        <v>0</v>
+        <v>1.0494</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>0.217</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>3.111</v>
       </c>
       <c r="I37">
-        <v>0</v>
+        <v>1.228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>